<commit_message>
feat: Restructure comprehensive PDF layouts and configure Vercel serverless build routes
</commit_message>
<xml_diff>
--- a/Site_Performance_Report.xlsx
+++ b/Site_Performance_Report.xlsx
@@ -490,7 +490,7 @@
     <t>Details</t>
   </si>
   <si>
-    <t>2026-06-28 18:11:45</t>
+    <t>2026-06-28 19:47:28</t>
   </si>
   <si>
     <t>Construction file</t>
@@ -505,18 +505,18 @@
     <t>Window frame</t>
   </si>
   <si>
+    <t>Possession</t>
+  </si>
+  <si>
     <t>Finishing Completion</t>
   </si>
   <si>
+    <t>Booking</t>
+  </si>
+  <si>
     <t>Agreement</t>
   </si>
   <si>
-    <t>Booking</t>
-  </si>
-  <si>
-    <t>Possession</t>
-  </si>
-  <si>
     <t>System</t>
   </si>
   <si>
@@ -532,16 +532,16 @@
     <t>Activity delayed by 25 days but 'Delay Reason' is missing.</t>
   </si>
   <si>
+    <t>Milestone Linked 'Possession' in Collections does not match any Activity in Construction Daily targets.</t>
+  </si>
+  <si>
     <t>Milestone Linked 'Finishing Completion' in Collections does not match any Activity in Construction Daily targets.</t>
   </si>
   <si>
+    <t>Milestone Linked 'Booking' in Collections does not match any Activity in Construction Daily targets.</t>
+  </si>
+  <si>
     <t>Milestone Linked 'Agreement' in Collections does not match any Activity in Construction Daily targets.</t>
-  </si>
-  <si>
-    <t>Milestone Linked 'Booking' in Collections does not match any Activity in Construction Daily targets.</t>
-  </si>
-  <si>
-    <t>Milestone Linked 'Possession' in Collections does not match any Activity in Construction Daily targets.</t>
   </si>
   <si>
     <t>'Customer Code'</t>

</xml_diff>